<commit_message>
Match UUID between the ODYM_t6_P5_torecycling parameter file and config file
</commit_message>
<xml_diff>
--- a/docs/Files/Tutorial6_JV_2/ODYM_T6_P5_ToRecycling_V1.0.xlsx
+++ b/docs/Files/Tutorial6_JV_2/ODYM_T6_P5_ToRecycling_V1.0.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28827"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC25FAEF-4984-4506-B7DB-E151B5EA0104}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B11B319C-E833-473A-9850-73CE46D738AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="3" r:id="rId1"/>
@@ -13,12 +13,25 @@
     <sheet name="log" sheetId="4" r:id="rId3"/>
     <sheet name="ref" sheetId="5" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="117">
   <si>
     <t>Format_Version</t>
   </si>
@@ -342,9 +355,6 @@
   </si>
   <si>
     <t>ODYM_T6_P5_ToRefurbishment</t>
-  </si>
-  <si>
-    <t>6213e899-8367-483a-8d09-a0c0831c22e8</t>
   </si>
   <si>
     <t>ODYM_T6_P5_ToRecycling</t>
@@ -841,7 +851,7 @@
         <v>18</v>
       </c>
       <c r="B3" s="16" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>16</v>
@@ -855,7 +865,7 @@
         <v>20</v>
       </c>
       <c r="B4" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>16</v>
@@ -939,7 +949,7 @@
         <v>25</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>16</v>
@@ -1258,7 +1268,7 @@
         <v>54</v>
       </c>
       <c r="I2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
@@ -1287,7 +1297,7 @@
         <v>54</v>
       </c>
       <c r="I3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
@@ -1316,7 +1326,7 @@
         <v>54</v>
       </c>
       <c r="I4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
@@ -1345,7 +1355,7 @@
         <v>54</v>
       </c>
       <c r="I5" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
@@ -1374,7 +1384,7 @@
         <v>54</v>
       </c>
       <c r="I6" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
@@ -1403,7 +1413,7 @@
         <v>54</v>
       </c>
       <c r="I7" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
@@ -1432,7 +1442,7 @@
         <v>54</v>
       </c>
       <c r="I8" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
@@ -1461,7 +1471,7 @@
         <v>54</v>
       </c>
       <c r="I9" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
@@ -1531,7 +1541,7 @@
       </c>
       <c r="E3" s="15"/>
       <c r="F3" s="12" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="G3" t="s">
         <v>89</v>
@@ -1596,8 +1606,9 @@
       </c>
     </row>
     <row r="3" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="B3" s="16" t="s">
-        <v>107</v>
+      <c r="B3" s="16" t="str">
+        <f>Cover!B3</f>
+        <v>ODYM_T6_P5_ToRecycling</v>
       </c>
       <c r="C3">
         <v>1</v>

</xml_diff>